<commit_message>
Daily EOD data and reports for 2026-10-14
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261014.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261014.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.745</v>
+        <v>1.742</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.028</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>267300.85</v>
+        <v>266841.3</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3829.52</v>
+        <v>-4289.07</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.415</v>
+        <v>2.41</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.045</v>
+        <v>-0.05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.83%</t>
+          <t>-2.03%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>169050</v>
+        <v>168700</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-3150</v>
+        <v>-3500</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>61.25</v>
+        <v>61.025</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.255</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>-0.42%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>490000</v>
+        <v>488200</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-240</v>
+        <v>-2040</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.005</v>
+        <v>0.001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>264.54</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-220.45</v>
+        <v>44.09</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>152.47</v>
+        <v>151.08</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-2.03</v>
+        <v>-3.42</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-1.31%</t>
+          <t>-2.21%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.005</v>
+        <v>-0.005</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.58%</t>
+          <t>-0.58%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8700</v>
+        <v>8600</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>50</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>183.09</v>
+        <v>184.14</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-1.49</v>
+        <v>-0.44</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.81%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>732360</v>
+        <v>736560</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-5960</v>
+        <v>-1760</v>
       </c>
     </row>
     <row r="11">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.093</v>
+        <v>0.091</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>-0.002</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-2.15%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>558</v>
+        <v>546</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.87</v>
+        <v>34.73</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.29</v>
+        <v>-0.43</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.82%</t>
+          <t>-1.22%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.89</v>
+        <v>32.99</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.11</v>
+        <v>0.21</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.34%</t>
+          <t>0.64%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42362.32</v>
+        <v>42491.12</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>141.68</v>
+        <v>270.48</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1754846.61</v>
+        <v>1756718.41</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-17067.22</v>
+        <v>-15195.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>